<commit_message>
merging file and updating the report
</commit_message>
<xml_diff>
--- a/shared/download/Export_Report.xlsx
+++ b/shared/download/Export_Report.xlsx
@@ -413,65 +413,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>Subject</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>File</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Folder</t>
+          <t>FilePath</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Carton Clean Up 04/26/2026</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Test one</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Merged</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>C:/Users/Renan Boniza/Desktop/Automation/daily-business-report/shared/download</t>
-        </is>
-      </c>
+          <t>C:/Users/Renan Boniza/Desktop/Automation/daily-business-report/shared/download\Carton_Clean_Up_04262026.xlsx</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Test One</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Test two</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
           <t>Received</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>C:/Users/Renan Boniza/Desktop/Automation/daily-business-report/shared/download</t>
@@ -479,24 +475,36 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Test Two</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Test three</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>C:/Users/Renan Boniza/Desktop/Automation/daily-business-report/shared/download</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Test Three</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>No Email Received</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>C:/Users/Renan Boniza/Desktop/Automation/daily-business-report/shared/download</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>